<commit_message>
Passage au template2 (#175)
* Revert "Revert "Feat/template2 (#173)" (#174)"

This reverts commit 8bd7b9d33d3ac6e9b59df57b103515acba302b85.

* Delete resources directory

* Delete input/resources directory

* Update sushi-config.yaml

* Update FRLMDoseNumber.fsh

* Update FRLMTechniqueImagerie.fsh 1a7ff52ac617ab738a9e0e9d1370ad3d6cd13e92
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-cda-accidents-transfusionnels.xlsx
+++ b/main/ig/StructureDefinition-fr-cda-accidents-transfusionnels.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3196" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3196" uniqueCount="340">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-29T12:53:00+00:00</t>
+    <t>2026-06-29T14:20:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -830,6 +830,10 @@
   </si>
   <si>
     <t>ED.thumbnail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ED-1:Thumbnails cannot contain their own thumbnails {thumbnail.empty()}
+</t>
   </si>
   <si>
     <t>Observation.statusCode</t>
@@ -7344,7 +7348,7 @@
         <v>74</v>
       </c>
       <c r="AJ58" t="s" s="2">
-        <v>74</v>
+        <v>266</v>
       </c>
       <c r="AK58" t="s" s="2">
         <v>74</v>
@@ -7352,10 +7356,10 @@
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -7381,10 +7385,10 @@
         <v>91</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
@@ -7415,7 +7419,7 @@
       </c>
       <c r="Y59" s="2"/>
       <c r="Z59" t="s" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="AA59" t="s" s="2">
         <v>74</v>
@@ -7433,7 +7437,7 @@
         <v>74</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>80</v>
@@ -7453,10 +7457,10 @@
     </row>
     <row r="60" hidden="true">
       <c r="A60" t="s" s="2">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -7554,10 +7558,10 @@
     </row>
     <row r="61" hidden="true">
       <c r="A61" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
@@ -7598,7 +7602,7 @@
         <v>74</v>
       </c>
       <c r="S61" t="s" s="2">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="T61" t="s" s="2">
         <v>74</v>
@@ -7657,10 +7661,10 @@
     </row>
     <row r="62" hidden="true">
       <c r="A62" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -7760,10 +7764,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -7863,10 +7867,10 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -7966,10 +7970,10 @@
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -8069,10 +8073,10 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -8170,10 +8174,10 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -8271,10 +8275,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -8374,10 +8378,10 @@
     </row>
     <row r="69" hidden="true">
       <c r="A69" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -8477,10 +8481,10 @@
     </row>
     <row r="70" hidden="true">
       <c r="A70" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -8580,10 +8584,10 @@
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -8606,13 +8610,13 @@
         <v>74</v>
       </c>
       <c r="K71" t="s" s="2">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="M71" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="N71" s="2"/>
       <c r="O71" s="2"/>
@@ -8663,7 +8667,7 @@
         <v>74</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>80</v>
@@ -8683,10 +8687,10 @@
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -8709,7 +8713,7 @@
         <v>74</v>
       </c>
       <c r="K72" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="L72" s="2"/>
       <c r="M72" s="2"/>
@@ -8742,7 +8746,7 @@
       </c>
       <c r="Y72" s="2"/>
       <c r="Z72" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="AA72" t="s" s="2">
         <v>74</v>
@@ -8760,7 +8764,7 @@
         <v>74</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>80</v>
@@ -8780,10 +8784,10 @@
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -8806,7 +8810,7 @@
         <v>74</v>
       </c>
       <c r="K73" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="L73" s="2"/>
       <c r="M73" s="2"/>
@@ -8859,7 +8863,7 @@
         <v>74</v>
       </c>
       <c r="AF73" t="s" s="2">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="AG73" t="s" s="2">
         <v>80</v>
@@ -8879,10 +8883,10 @@
     </row>
     <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -8938,25 +8942,25 @@
       </c>
       <c r="Y74" s="2"/>
       <c r="Z74" t="s" s="2">
+        <v>291</v>
+      </c>
+      <c r="AA74" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AB74" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AC74" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD74" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AE74" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AF74" t="s" s="2">
         <v>290</v>
-      </c>
-      <c r="AA74" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB74" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC74" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD74" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE74" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF74" t="s" s="2">
-        <v>289</v>
       </c>
       <c r="AG74" t="s" s="2">
         <v>80</v>
@@ -8976,10 +8980,10 @@
     </row>
     <row r="75">
       <c r="A75" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -9005,10 +9009,10 @@
         <v>221</v>
       </c>
       <c r="L75" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="M75" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="N75" s="2"/>
       <c r="O75" s="2"/>
@@ -9059,7 +9063,7 @@
         <v>74</v>
       </c>
       <c r="AF75" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="AG75" t="s" s="2">
         <v>80</v>
@@ -9079,10 +9083,10 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -9105,7 +9109,7 @@
         <v>74</v>
       </c>
       <c r="K76" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="L76" s="2"/>
       <c r="M76" s="2"/>
@@ -9138,25 +9142,25 @@
       </c>
       <c r="Y76" s="2"/>
       <c r="Z76" t="s" s="2">
+        <v>295</v>
+      </c>
+      <c r="AA76" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AB76" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AC76" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD76" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AE76" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AF76" t="s" s="2">
         <v>294</v>
-      </c>
-      <c r="AA76" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB76" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC76" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD76" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE76" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF76" t="s" s="2">
-        <v>293</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>80</v>
@@ -9176,10 +9180,10 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -9202,7 +9206,7 @@
         <v>74</v>
       </c>
       <c r="K77" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="L77" s="2"/>
       <c r="M77" s="2"/>
@@ -9235,25 +9239,25 @@
       </c>
       <c r="Y77" s="2"/>
       <c r="Z77" t="s" s="2">
+        <v>297</v>
+      </c>
+      <c r="AA77" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AB77" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AC77" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AD77" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AE77" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="AF77" t="s" s="2">
         <v>296</v>
-      </c>
-      <c r="AA77" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB77" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC77" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD77" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE77" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF77" t="s" s="2">
-        <v>295</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>80</v>
@@ -9273,10 +9277,10 @@
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -9303,7 +9307,7 @@
       </c>
       <c r="L78" s="2"/>
       <c r="M78" t="s" s="2">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="N78" s="2"/>
       <c r="O78" s="2"/>
@@ -9354,7 +9358,7 @@
         <v>74</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>80</v>
@@ -9374,10 +9378,10 @@
     </row>
     <row r="79" hidden="true">
       <c r="A79" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -9400,7 +9404,7 @@
         <v>74</v>
       </c>
       <c r="K79" t="s" s="2">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="L79" s="2"/>
       <c r="M79" s="2"/>
@@ -9453,7 +9457,7 @@
         <v>74</v>
       </c>
       <c r="AF79" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="AG79" t="s" s="2">
         <v>80</v>
@@ -9473,10 +9477,10 @@
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -9499,7 +9503,7 @@
         <v>74</v>
       </c>
       <c r="K80" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="L80" s="2"/>
       <c r="M80" s="2"/>
@@ -9552,7 +9556,7 @@
         <v>74</v>
       </c>
       <c r="AF80" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="AG80" t="s" s="2">
         <v>80</v>
@@ -9572,10 +9576,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -9598,7 +9602,7 @@
         <v>74</v>
       </c>
       <c r="K81" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L81" s="2"/>
       <c r="M81" s="2"/>
@@ -9651,7 +9655,7 @@
         <v>74</v>
       </c>
       <c r="AF81" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="AG81" t="s" s="2">
         <v>80</v>
@@ -9671,10 +9675,10 @@
     </row>
     <row r="82" hidden="true">
       <c r="A82" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -9697,13 +9701,13 @@
         <v>74</v>
       </c>
       <c r="K82" t="s" s="2">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="L82" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="M82" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="N82" s="2"/>
       <c r="O82" s="2"/>
@@ -9754,7 +9758,7 @@
         <v>74</v>
       </c>
       <c r="AF82" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="AG82" t="s" s="2">
         <v>80</v>
@@ -9774,10 +9778,10 @@
     </row>
     <row r="83" hidden="true">
       <c r="A83" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -9800,7 +9804,7 @@
         <v>74</v>
       </c>
       <c r="K83" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="L83" s="2"/>
       <c r="M83" s="2"/>
@@ -9853,7 +9857,7 @@
         <v>74</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>80</v>
@@ -9873,10 +9877,10 @@
     </row>
     <row r="84" hidden="true">
       <c r="A84" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -9899,7 +9903,7 @@
         <v>74</v>
       </c>
       <c r="K84" t="s" s="2">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="L84" s="2"/>
       <c r="M84" s="2"/>
@@ -9952,7 +9956,7 @@
         <v>74</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>80</v>
@@ -9972,10 +9976,10 @@
     </row>
     <row r="85" hidden="true">
       <c r="A85" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -9998,7 +10002,7 @@
         <v>74</v>
       </c>
       <c r="K85" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="L85" s="2"/>
       <c r="M85" s="2"/>
@@ -10051,7 +10055,7 @@
         <v>74</v>
       </c>
       <c r="AF85" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="AG85" t="s" s="2">
         <v>80</v>
@@ -10071,10 +10075,10 @@
     </row>
     <row r="86" hidden="true">
       <c r="A86" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -10097,7 +10101,7 @@
         <v>74</v>
       </c>
       <c r="K86" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="L86" s="2"/>
       <c r="M86" s="2"/>
@@ -10150,7 +10154,7 @@
         <v>74</v>
       </c>
       <c r="AF86" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="AG86" t="s" s="2">
         <v>80</v>
@@ -10170,10 +10174,10 @@
     </row>
     <row r="87" hidden="true">
       <c r="A87" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -10196,7 +10200,7 @@
         <v>74</v>
       </c>
       <c r="K87" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="L87" s="2"/>
       <c r="M87" s="2"/>
@@ -10249,7 +10253,7 @@
         <v>74</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>80</v>
@@ -10269,10 +10273,10 @@
     </row>
     <row r="88" hidden="true">
       <c r="A88" t="s" s="2">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -10295,7 +10299,7 @@
         <v>74</v>
       </c>
       <c r="K88" t="s" s="2">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="L88" s="2"/>
       <c r="M88" s="2"/>
@@ -10348,7 +10352,7 @@
         <v>74</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>80</v>
@@ -10368,10 +10372,10 @@
     </row>
     <row r="89" hidden="true">
       <c r="A89" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -10394,11 +10398,11 @@
         <v>74</v>
       </c>
       <c r="K89" t="s" s="2">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="L89" s="2"/>
       <c r="M89" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="N89" s="2"/>
       <c r="O89" s="2"/>
@@ -10449,7 +10453,7 @@
         <v>74</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>80</v>
@@ -10469,10 +10473,10 @@
     </row>
     <row r="90" hidden="true">
       <c r="A90" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -10570,10 +10574,10 @@
     </row>
     <row r="91" hidden="true">
       <c r="A91" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -10671,10 +10675,10 @@
     </row>
     <row r="92" hidden="true">
       <c r="A92" t="s" s="2">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -10772,10 +10776,10 @@
     </row>
     <row r="93" hidden="true">
       <c r="A93" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -10873,10 +10877,10 @@
     </row>
     <row r="94" hidden="true">
       <c r="A94" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -10976,10 +10980,10 @@
     </row>
     <row r="95" hidden="true">
       <c r="A95" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -11079,10 +11083,10 @@
     </row>
     <row r="96" hidden="true">
       <c r="A96" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -11182,10 +11186,10 @@
     </row>
     <row r="97" hidden="true">
       <c r="A97" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -11285,10 +11289,10 @@
     </row>
     <row r="98" hidden="true">
       <c r="A98" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -11386,10 +11390,10 @@
     </row>
     <row r="99" hidden="true">
       <c r="A99" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -11423,7 +11427,7 @@
       </c>
       <c r="Q99" s="2"/>
       <c r="R99" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="S99" t="s" s="2">
         <v>74</v>
@@ -11445,7 +11449,7 @@
       </c>
       <c r="Y99" s="2"/>
       <c r="Z99" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="AA99" t="s" s="2">
         <v>74</v>
@@ -11463,7 +11467,7 @@
         <v>74</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>80</v>
@@ -11483,10 +11487,10 @@
     </row>
     <row r="100" hidden="true">
       <c r="A100" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -11509,7 +11513,7 @@
         <v>74</v>
       </c>
       <c r="K100" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="L100" s="2"/>
       <c r="M100" s="2"/>
@@ -11562,7 +11566,7 @@
         <v>74</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>75</v>
@@ -11582,10 +11586,10 @@
     </row>
     <row r="101" hidden="true">
       <c r="A101" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B101" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C101" s="2"/>
       <c r="D101" t="s" s="2">
@@ -11608,7 +11612,7 @@
         <v>74</v>
       </c>
       <c r="K101" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="L101" s="2"/>
       <c r="M101" s="2"/>
@@ -11661,7 +11665,7 @@
         <v>74</v>
       </c>
       <c r="AF101" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="AG101" t="s" s="2">
         <v>80</v>

</xml_diff>